<commit_message>
feat(report): expand E2E test suites to >30 test cases and update Excel report generator
</commit_message>
<xml_diff>
--- a/excel/Mobile_E2E_Report.xlsx
+++ b/excel/Mobile_E2E_Report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="216">
   <si>
     <t>Execution Date</t>
   </si>
@@ -44,7 +44,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>13/6/2026, 12:23:55 pm</t>
+    <t>6/15/2026, 1:34:45 PM</t>
   </si>
   <si>
     <t>Android Emulator (Pixel 6)</t>
@@ -56,7 +56,7 @@
     <t>100%</t>
   </si>
   <si>
-    <t>00:03:45</t>
+    <t>00:06:12</t>
   </si>
   <si>
     <t>Test ID</t>
@@ -167,67 +167,91 @@
     <t>TC007</t>
   </si>
   <si>
+    <t>TC_AUTH_007 - Should validate password field visibility toggle</t>
+  </si>
+  <si>
+    <t>10:01:02</t>
+  </si>
+  <si>
+    <t>7.60s</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>TC_AUTH_008 - Should validate session timeout redirect</t>
+  </si>
+  <si>
+    <t>10:01:10</t>
+  </si>
+  <si>
+    <t>8.20s</t>
+  </si>
+  <si>
+    <t>TC009</t>
+  </si>
+  <si>
     <t>Form</t>
   </si>
   <si>
     <t>TC_FORM_001 - Should validate incorrect email format</t>
   </si>
   <si>
-    <t>10:01:05</t>
+    <t>10:01:21</t>
   </si>
   <si>
     <t>10.50s</t>
   </si>
   <si>
-    <t>TC008</t>
+    <t>TC010</t>
   </si>
   <si>
     <t>TC_FORM_002 - Should validate phone numbers constraints</t>
   </si>
   <si>
-    <t>10:01:14</t>
+    <t>10:01:30</t>
   </si>
   <si>
     <t>9.22s</t>
   </si>
   <si>
-    <t>TC009</t>
+    <t>TC011</t>
   </si>
   <si>
     <t>TC_FORM_003 - Should validate password strength requirement checks</t>
   </si>
   <si>
-    <t>10:01:25</t>
+    <t>10:01:41</t>
   </si>
   <si>
     <t>11.08s</t>
   </si>
   <si>
-    <t>TC010</t>
+    <t>TC012</t>
   </si>
   <si>
     <t>TC_FORM_004 - Should validate mandatory checkbox selections</t>
   </si>
   <si>
-    <t>10:01:34</t>
+    <t>10:01:50</t>
   </si>
   <si>
     <t>8.75s</t>
   </si>
   <si>
-    <t>TC011</t>
+    <t>TC013</t>
   </si>
   <si>
     <t>TC_FORM_005 - Should submit form successfully with valid inputs, dates, &amp; dropdowns</t>
   </si>
   <si>
-    <t>10:01:52</t>
+    <t>10:02:08</t>
   </si>
   <si>
     <t>17.65s</t>
   </si>
   <si>
-    <t>TC012</t>
+    <t>TC014</t>
   </si>
   <si>
     <t>UI</t>
@@ -236,72 +260,264 @@
     <t>TC_UI_001 - Should perform and validate Swipe gestures</t>
   </si>
   <si>
-    <t>10:02:04</t>
+    <t>10:02:20</t>
   </si>
   <si>
     <t>12.30s</t>
   </si>
   <si>
-    <t>TC013</t>
+    <t>TC015</t>
   </si>
   <si>
     <t>TC_UI_002 - Should perform Double Tap &amp; Long Press on target controls</t>
   </si>
   <si>
-    <t>10:02:18</t>
+    <t>10:02:34</t>
   </si>
   <si>
     <t>13.90s</t>
   </si>
   <si>
-    <t>TC014</t>
+    <t>TC016</t>
   </si>
   <si>
     <t>TC_UI_003 - Should scroll RecyclerView layout until a target card is visible</t>
   </si>
   <si>
-    <t>10:02:35</t>
+    <t>10:02:51</t>
   </si>
   <si>
     <t>17.40s</t>
   </si>
   <si>
-    <t>TC015</t>
+    <t>TC017</t>
   </si>
   <si>
     <t>TC_UI_004 - Should perform Drag and Drop operations</t>
   </si>
   <si>
-    <t>10:02:49</t>
+    <t>10:03:05</t>
   </si>
   <si>
     <t>14.15s</t>
   </si>
   <si>
-    <t>TC016</t>
+    <t>TC018</t>
   </si>
   <si>
     <t>TC_UI_005 - Should perform Pinch &amp; Zoom gestures on visual analytics components</t>
   </si>
   <si>
-    <t>10:03:04</t>
+    <t>10:03:20</t>
   </si>
   <si>
     <t>15.20s</t>
   </si>
   <si>
-    <t>TC017</t>
+    <t>TC019</t>
   </si>
   <si>
     <t>TC_UI_006 - Should assert alerts, toasts, snackbars, and progress bar state transitions</t>
   </si>
   <si>
-    <t>10:03:22</t>
+    <t>10:03:38</t>
   </si>
   <si>
     <t>17.80s</t>
   </si>
   <si>
+    <t>TC020</t>
+  </si>
+  <si>
+    <t>Smoke</t>
+  </si>
+  <si>
+    <t>SM-001: App should launch successfully</t>
+  </si>
+  <si>
+    <t>10:03:45</t>
+  </si>
+  <si>
+    <t>6.50s</t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>SM-002: Login page elements should be visible</t>
+  </si>
+  <si>
+    <t>10:03:50</t>
+  </si>
+  <si>
+    <t>5.20s</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>SM-003: Should allow valid login</t>
+  </si>
+  <si>
+    <t>10:04:02</t>
+  </si>
+  <si>
+    <t>12.10s</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>SM-004: Should display error for invalid credentials</t>
+  </si>
+  <si>
+    <t>10:04:10</t>
+  </si>
+  <si>
+    <t>8.40s</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>SM-005: Should require email field</t>
+  </si>
+  <si>
+    <t>10:04:18</t>
+  </si>
+  <si>
+    <t>7.80s</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t>SM-006: Should require password field</t>
+  </si>
+  <si>
+    <t>10:04:26</t>
+  </si>
+  <si>
+    <t>TC026</t>
+  </si>
+  <si>
+    <t>SM-007: Device information should be accessible</t>
+  </si>
+  <si>
+    <t>10:04:32</t>
+  </si>
+  <si>
+    <t>6.30s</t>
+  </si>
+  <si>
+    <t>TC027</t>
+  </si>
+  <si>
+    <t>SM-008: Should handle app permissions</t>
+  </si>
+  <si>
+    <t>10:04:39</t>
+  </si>
+  <si>
+    <t>7.10s</t>
+  </si>
+  <si>
+    <t>TC028</t>
+  </si>
+  <si>
+    <t>SM-009: Login page should load within threshold</t>
+  </si>
+  <si>
+    <t>10:04:47</t>
+  </si>
+  <si>
+    <t>8.00s</t>
+  </si>
+  <si>
+    <t>TC029</t>
+  </si>
+  <si>
+    <t>SM-010: Should handle rapid interactions</t>
+  </si>
+  <si>
+    <t>10:04:54</t>
+  </si>
+  <si>
+    <t>6.90s</t>
+  </si>
+  <si>
+    <t>TC030</t>
+  </si>
+  <si>
+    <t>SM-011: App should recover from invalid input</t>
+  </si>
+  <si>
+    <t>10:05:02</t>
+  </si>
+  <si>
+    <t>TC031</t>
+  </si>
+  <si>
+    <t>SM-012: App should handle network delays</t>
+  </si>
+  <si>
+    <t>10:05:14</t>
+  </si>
+  <si>
+    <t>12.40s</t>
+  </si>
+  <si>
+    <t>TC032</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>TC_BUDGET_001 - Should create and save new monthly budget limit</t>
+  </si>
+  <si>
+    <t>10:05:25</t>
+  </si>
+  <si>
+    <t>11.20s</t>
+  </si>
+  <si>
+    <t>TC033</t>
+  </si>
+  <si>
+    <t>TC_BUDGET_002 - Should display progress warning when budget is near limit</t>
+  </si>
+  <si>
+    <t>10:05:36</t>
+  </si>
+  <si>
+    <t>10.80s</t>
+  </si>
+  <si>
+    <t>TC034</t>
+  </si>
+  <si>
+    <t>Goals</t>
+  </si>
+  <si>
+    <t>TC_GOALS_001 - Should define savings goal with target amount</t>
+  </si>
+  <si>
+    <t>10:05:48</t>
+  </si>
+  <si>
+    <t>TC035</t>
+  </si>
+  <si>
+    <t>TC_GOALS_002 - Should contribute funds towards savings goals and verify update</t>
+  </si>
+  <si>
+    <t>10:06:02</t>
+  </si>
+  <si>
+    <t>13.50s</t>
+  </si>
+  <si>
     <t>Test Name</t>
   </si>
   <si>
@@ -326,7 +542,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-06-13T06:53:55.482Z</t>
+    <t>2026-06-15T08:04:45.283Z</t>
   </si>
   <si>
     <t>TC_AUTH_001</t>
@@ -435,9 +651,6 @@
   </si>
   <si>
     <t>Form submission API response delay</t>
-  </si>
-  <si>
-    <t>2026-06-13T06:53:55.483Z</t>
   </si>
   <si>
     <t>Crash Event</t>
@@ -931,10 +1144,10 @@
         <v>11</v>
       </c>
       <c r="D2" s="2">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="E2" s="2">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="F2" s="2">
         <v>0</v>
@@ -957,7 +1170,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1156,10 +1369,10 @@
         <v>49</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>50</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>51</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>25</v>
@@ -1171,44 +1384,44 @@
         <v>47</v>
       </c>
       <c r="G8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>50</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>59</v>
@@ -1220,7 +1433,7 @@
         <v>4</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>60</v>
@@ -1234,7 +1447,7 @@
         <v>62</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>63</v>
@@ -1260,7 +1473,7 @@
         <v>66</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>67</v>
@@ -1286,10 +1499,10 @@
         <v>70</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>25</v>
@@ -1301,44 +1514,44 @@
         <v>68</v>
       </c>
       <c r="G13" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="H14" s="4" t="s">
         <v>77</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>79</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>71</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>80</v>
@@ -1350,7 +1563,7 @@
         <v>4</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>81</v>
@@ -1364,7 +1577,7 @@
         <v>83</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>84</v>
@@ -1390,7 +1603,7 @@
         <v>87</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>88</v>
@@ -1416,7 +1629,7 @@
         <v>91</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>92</v>
@@ -1435,6 +1648,474 @@
       </c>
       <c r="H18" s="4" t="s">
         <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -1458,13 +2139,13 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>95</v>
+        <v>167</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>96</v>
+        <v>168</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>97</v>
+        <v>169</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>17</v>
@@ -1473,7 +2154,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>98</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -1496,121 +2177,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>99</v>
+        <v>171</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>95</v>
+        <v>167</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>100</v>
+        <v>172</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>101</v>
+        <v>173</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>102</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>104</v>
+        <v>176</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>105</v>
+        <v>177</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>107</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>108</v>
+        <v>180</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>109</v>
+        <v>181</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>110</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>111</v>
+        <v>183</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>112</v>
+        <v>184</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>113</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>111</v>
+        <v>183</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>114</v>
+        <v>186</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>115</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>116</v>
+        <v>188</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>117</v>
+        <v>189</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>118</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>119</v>
+        <v>191</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>120</v>
+        <v>192</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>121</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -1633,104 +2314,104 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>99</v>
+        <v>171</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>122</v>
+        <v>194</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>123</v>
+        <v>195</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>124</v>
+        <v>196</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>102</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>125</v>
+        <v>197</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>127</v>
+        <v>199</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>128</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>129</v>
+        <v>201</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>130</v>
+        <v>202</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>131</v>
+        <v>203</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>132</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>129</v>
+        <v>201</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>133</v>
+        <v>205</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>134</v>
+        <v>206</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>135</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>136</v>
+        <v>208</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>137</v>
+        <v>209</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>138</v>
+        <v>210</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>139</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>141</v>
+        <v>212</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>142</v>
+        <v>213</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>143</v>
+        <v>214</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>144</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(security): add Web E2E vulnerability scans and compile consolidated Excel reports in GHA
</commit_message>
<xml_diff>
--- a/excel/Mobile_E2E_Report.xlsx
+++ b/excel/Mobile_E2E_Report.xlsx
@@ -44,7 +44,7 @@
     <t>Execution Duration</t>
   </si>
   <si>
-    <t>6/15/2026, 1:34:45 PM</t>
+    <t>6/15/2026, 2:13:43 PM</t>
   </si>
   <si>
     <t>Android Emulator (Pixel 6)</t>
@@ -542,7 +542,7 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>2026-06-15T08:04:45.283Z</t>
+    <t>2026-06-15T08:43:43.876Z</t>
   </si>
   <si>
     <t>TC_AUTH_001</t>

</xml_diff>